<commit_message>
saves moves correctly ! phew
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/306EJan1808.xlsx
+++ b/Austerlitz/Turns/306EJan1808.xlsx
@@ -7137,13 +7137,41 @@
       <c r="A215" s="4">
         <v>1</v>
       </c>
-      <c r="B215" s="17"/>
-      <c r="C215" s="10"/>
-      <c r="D215" s="10"/>
-      <c r="E215" s="10"/>
-      <c r="F215" s="10"/>
-      <c r="G215" s="10"/>
-      <c r="H215" s="10"/>
+      <c r="B215" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C215" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D215" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E215" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F215" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G215" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H215" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I215" s="4"/>
       <c r="J215" s="4"/>
       <c r="K215" s="5"/>
@@ -7199,7 +7227,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="216">
       <c r="A216" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B216" s="10"/>
       <c r="C216" s="10"/>
@@ -7263,16 +7291,16 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="217">
       <c r="A217" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B217" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C217" s="10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D217" s="10" t="inlineStr">
@@ -7282,7 +7310,7 @@
       </c>
       <c r="E217" s="10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F217" s="10" t="inlineStr">
@@ -7292,12 +7320,12 @@
       </c>
       <c r="G217" s="10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H217" s="10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I217" s="4"/>
@@ -7355,11 +7383,11 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="218">
       <c r="A218" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B218" s="10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C218" s="10" t="inlineStr">
@@ -7382,8 +7410,16 @@
           <t>2</t>
         </is>
       </c>
-      <c r="G218" s="10"/>
-      <c r="H218" s="10"/>
+      <c r="G218" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H218" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I218" s="4"/>
       <c r="J218" s="4"/>
       <c r="K218" s="5"/>
@@ -7439,7 +7475,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="219">
       <c r="A219" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B219" s="10"/>
       <c r="C219" s="10"/>
@@ -7503,7 +7539,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="220">
       <c r="A220" s="4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B220" s="10"/>
       <c r="C220" s="10"/>
@@ -7567,7 +7603,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="221">
       <c r="A221" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B221" s="10"/>
       <c r="C221" s="10"/>
@@ -7631,7 +7667,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="222">
       <c r="A222" s="4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B222" s="10"/>
       <c r="C222" s="10"/>
@@ -7695,7 +7731,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="223">
       <c r="A223" s="4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B223" s="10"/>
       <c r="C223" s="10"/>
@@ -7759,7 +7795,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="224">
       <c r="A224" s="4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B224" s="10"/>
       <c r="C224" s="17"/>
@@ -7823,7 +7859,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="225">
       <c r="A225" s="4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B225" s="10"/>
       <c r="C225" s="10"/>
@@ -7887,7 +7923,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="226">
       <c r="A226" s="4">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B226" s="10"/>
       <c r="C226" s="10"/>
@@ -7951,7 +7987,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="227">
       <c r="A227" s="4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B227" s="10"/>
       <c r="C227" s="10"/>
@@ -8015,7 +8051,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="228">
       <c r="A228" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B228" s="10"/>
       <c r="C228" s="10"/>
@@ -8079,7 +8115,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="229">
       <c r="A229" s="4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B229" s="10"/>
       <c r="C229" s="10"/>
@@ -8143,7 +8179,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="230">
       <c r="A230" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B230" s="10"/>
       <c r="C230" s="10"/>
@@ -8207,7 +8243,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="231">
       <c r="A231" s="4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B231" s="10"/>
       <c r="C231" s="10"/>
@@ -8271,7 +8307,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="232">
       <c r="A232" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B232" s="10"/>
       <c r="C232" s="10"/>
@@ -8335,7 +8371,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="233">
       <c r="A233" s="4">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B233" s="10"/>
       <c r="C233" s="10"/>
@@ -8399,7 +8435,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="234">
       <c r="A234" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B234" s="10"/>
       <c r="C234" s="10"/>
@@ -8463,7 +8499,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="235">
       <c r="A235" s="4">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B235" s="10"/>
       <c r="C235" s="10"/>
@@ -8527,7 +8563,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="236">
       <c r="A236" s="4">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B236" s="10"/>
       <c r="C236" s="10"/>
@@ -8591,7 +8627,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="237">
       <c r="A237" s="4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B237" s="10"/>
       <c r="C237" s="10"/>
@@ -8655,7 +8691,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="238">
       <c r="A238" s="4">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B238" s="10"/>
       <c r="C238" s="10"/>
@@ -8719,7 +8755,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="239">
       <c r="A239" s="4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B239" s="10"/>
       <c r="C239" s="10"/>
@@ -8783,7 +8819,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="240">
       <c r="A240" s="4">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B240" s="10"/>
       <c r="C240" s="10"/>
@@ -8847,7 +8883,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="241">
       <c r="A241" s="4">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B241" s="10"/>
       <c r="C241" s="10"/>
@@ -8911,7 +8947,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="242">
       <c r="A242" s="4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B242" s="10"/>
       <c r="C242" s="10"/>
@@ -8975,7 +9011,7 @@
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="243">
       <c r="A243" s="4">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B243" s="10"/>
       <c r="C243" s="10"/>
@@ -9102,11 +9138,7 @@
       </c>
     </row>
     <row spans="1:12" ht="13.5" customHeight="1" outlineLevel="0" r="245">
-      <c r="A245" s="4" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
+      <c r="A245" s="4"/>
       <c r="B245" s="4"/>
       <c r="C245" s="4"/>
       <c r="D245" s="4"/>

</xml_diff>